<commit_message>
Open-gaps ledger closed: all 9 NW gaps verified against the code with the test that pins each
The ledger had sat at 9 OPEN while the commits claimed the fixes — exactly the docs-lag-reality
trap. Each row is now re-checked against the live source and carries its evidence: the
re-classification migration for stored CDs and money-market funds, the duplicate Cash heading, the
band/row right edge, the pill order, the dated hero band, the retirement wording, the since-line, and
the cushion (which also divided by a different cash figure than the group above it until yesterday).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mockups/NW-Performance-Mockup Finals - August 10/OPEN-GAPS-and-audit-method-2026-08-10.xlsx
+++ b/mockups/NW-Performance-Mockup Finals - August 10/OPEN-GAPS-and-audit-method-2026-08-10.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,8 +30,13 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -41,6 +46,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00854F0B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00085041"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DFF2E9"/>
       </patternFill>
     </fill>
   </fills>
@@ -56,10 +71,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -427,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -436,6 +455,7 @@
     <col width="58" customWidth="1" min="4" max="4"/>
     <col width="58" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="90" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -469,274 +489,324 @@
           <t>Status</t>
         </is>
       </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Verified against the CODE (2026-08-11)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>Founder</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>NW main</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>E*TRADE CD still shows under Cash</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>DATA REALITY — the cash-only rule was applied to NEW data only; existing/synced accounts were never re-classified</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>OPEN</t>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>CLOSED — a one-time re-classification runs over ALREADY-STORED accounts (store.runReclassifyOnce, called from Home on mount; reclassifyAccounts + RECLASSIFY_VERSION, idempotent). Test: 'a stored CD leaves Cash for Bonds'. A connected account that sends no holdings also keeps its own class now (fixed 2026-08-10), which was the same defect one layer down.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Founder</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>NW main</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>VMFXX (money-market fund) still under Cash</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>same class as #1 — needs a one-time migration over existing accounts</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>OPEN</t>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>CLOSED — same migration; test: 'VMFXX leaves Cash for Stocks'. Positions INSIDE an account are re-classified too, not just the account row.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Founder</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>NW main</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Inside the Cash group there is a SECOND "Cash" sub-heading with the items under it</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>NESTING — group bar and class sub-band duplicate each other</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>OPEN</t>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>CLOSED — a lone class matching its group renders its accounts directly (no repeated heading). Test: 'nesting: no class header repeats its own group name' asserts zero bare 'Cash' headers.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Founder</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>NW main</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>Group totals sit slightly LEFT of the row numbers</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>ALIGNMENT — band value inset differs from row value inset</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>OPEN</t>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>CLOSED — fixed structurally, not nudged: the whole own/owe list became one flat table where EVERY row (bands included) reserves the same 16pt arrow column. Test measures the rendered right inset of a section total, a group total, a class total and an account amount and asserts they agree.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Founder</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>NW main</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>"By category / By institution" pills sit BELOW What you owe; the mock puts them above the lists</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>ORDER</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>OPEN</t>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>CLOSED — pills render above the lists. Test: 'order: the grouping pills render BEFORE the WHAT YOU OWN band'.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="A7" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Claude</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>NW main</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>Hero band reads "YOUR NET WORTH"; mock reads "YOUR NET WORTH · AUG 4, 2026 info-dot"</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>TEXT DIFF</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>OPEN</t>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>CLOSED — the band reads 'YOUR NET WORTH · AUG 11, 2026' (today's date restored at the founder's ask 2026-08-11). Test asserts the dated title AND that today appears exactly once on the screen.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>Claude</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>NW main</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>Retirement card still uses the OLD "path ahead ... by 92" wording, unbanded; mock has the banded card with the approved sentence</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>TEXT DIFF + approved-words decision not applied here</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>OPEN</t>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>CLOSED — the card speaks the Plan hub's own sentence via onCourseSentence + lensChanceWord, with its info dot. Test: the retirement-card block in NetWorthScreen.test.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
+      <c r="A9" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>Claude</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>NW main</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>Under the change: code shows "as of Aug 10"; mock shows "since Aug 3, 2026"</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>TEXT DIFF — different meaning</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>OPEN</t>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>CLOSED — the line reads 'since Aug 3, 2026' (the true measured-from day, with the year), and the title's date is a separate fact (as-of today). Test: 'hero: today stamps the title, the since line carries the measured-from day'.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
+      <c r="A10" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>Claude</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>NW main</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>Emergency cushion card differs between the with-data screen and the mock</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>TEXT/STRUCTURE</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>OPEN</t>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>CLOSED — one cushion card in both states: 2.0 months + Tight ⚠ + the math line, and a progress bar (founder Q6). It also divides by the SAME cash the CASH group shows, which it did not before (it read $8,000 against a group of $8,838).</t>
         </is>
       </c>
     </row>

</xml_diff>